<commit_message>
feat(shift-schedule): expand month format support in Excel import
parseMonthYear now accepts: 'Jul 2025', 'Jul 25', 'Jul-25',
'07-2025', '07-25', 'July 2025', 'July 25', '2025-07', '07/2025'.
2-digit years resolved via y2k (+ 2000). 4-digit patterns checked
first to avoid ambiguity with 2-digit variants.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/shift_schedule_import_sample.xlsx
+++ b/docs/shift_schedule_import_sample.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10525"/>
-  <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/kuliah/hris-backend/docs/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{302FDEC7-C84F-C148-A141-8069935C448C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="19260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -25,13 +19,10 @@
     <t>Nama</t>
   </si>
   <si>
-    <t>month (contoh: Jan)</t>
+    <t>Jul 2025</t>
   </si>
   <si>
     <t>User A</t>
-  </si>
-  <si>
-    <t>User B</t>
   </si>
   <si>
     <t>pagi</t>
@@ -45,20 +36,32 @@
   <si>
     <t>libur</t>
   </si>
+  <si>
+    <t>User B</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -71,7 +74,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -83,27 +93,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="11">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -114,10 +144,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -155,71 +185,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -243,54 +273,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -300,7 +329,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -309,7 +338,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -318,7 +347,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -326,10 +355,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -358,7 +387,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -371,13 +400,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -395,15 +423,49 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CE4507C-3C21-C942-950C-4DD0B266065A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
   <dimension ref="A1:AF4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="54.5" customWidth="1"/>
+    <col min="1" max="1" style="9" width="54.57642857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="27" max="27" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="28" max="28" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="29" max="29" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="30" max="30" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="31" max="31" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="32" max="32" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -440,155 +502,204 @@
       <c r="AE1" s="3"/>
       <c r="AF1" s="3"/>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-      <c r="B2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
+      <c r="A2" s="4"/>
+      <c r="B2" s="5">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="5">
         <v>2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="5">
         <v>3</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="5">
         <v>4</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <v>5</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="5">
         <v>6</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5">
         <v>7</v>
       </c>
-      <c r="I2">
+      <c r="I2" s="5">
         <v>8</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="5">
         <v>9</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="5">
         <v>10</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="5">
         <v>11</v>
       </c>
-      <c r="M2">
+      <c r="M2" s="5">
         <v>12</v>
       </c>
-      <c r="N2">
+      <c r="N2" s="5">
         <v>13</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="5">
         <v>14</v>
       </c>
-      <c r="P2">
+      <c r="P2" s="5">
         <v>15</v>
       </c>
-      <c r="Q2">
+      <c r="Q2" s="5">
         <v>16</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="5">
         <v>17</v>
       </c>
-      <c r="S2">
+      <c r="S2" s="5">
         <v>18</v>
       </c>
-      <c r="T2">
+      <c r="T2" s="5">
         <v>19</v>
       </c>
-      <c r="U2">
+      <c r="U2" s="5">
         <v>20</v>
       </c>
-      <c r="V2">
+      <c r="V2" s="5">
         <v>21</v>
       </c>
-      <c r="W2">
+      <c r="W2" s="5">
         <v>22</v>
       </c>
-      <c r="X2">
+      <c r="X2" s="5">
         <v>23</v>
       </c>
-      <c r="Y2">
+      <c r="Y2" s="5">
         <v>24</v>
       </c>
-      <c r="Z2">
+      <c r="Z2" s="5">
         <v>25</v>
       </c>
-      <c r="AA2">
+      <c r="AA2" s="5">
         <v>26</v>
       </c>
-      <c r="AB2">
+      <c r="AB2" s="5">
         <v>27</v>
       </c>
-      <c r="AC2">
+      <c r="AC2" s="5">
         <v>28</v>
       </c>
-      <c r="AD2">
+      <c r="AD2" s="5">
         <v>29</v>
       </c>
-      <c r="AE2">
+      <c r="AE2" s="5">
         <v>30</v>
       </c>
-      <c r="AF2">
+      <c r="AF2" s="5">
         <v>31</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="F3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="H3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="I3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+      <c r="Q3" s="8"/>
+      <c r="R3" s="8"/>
+      <c r="S3" s="8"/>
+      <c r="T3" s="8"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="8"/>
+      <c r="W3" s="8"/>
+      <c r="X3" s="8"/>
+      <c r="Y3" s="8"/>
+      <c r="Z3" s="8"/>
+      <c r="AA3" s="8"/>
+      <c r="AB3" s="8"/>
+      <c r="AC3" s="8"/>
+      <c r="AD3" s="8"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+      <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>4</v>
-      </c>
+      <c r="F4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="8"/>
+      <c r="W4" s="8"/>
+      <c r="X4" s="8"/>
+      <c r="Y4" s="8"/>
+      <c r="Z4" s="8"/>
+      <c r="AA4" s="8"/>
+      <c r="AB4" s="8"/>
+      <c r="AC4" s="8"/>
+      <c r="AD4" s="8"/>
+      <c r="AE4" s="8"/>
+      <c r="AF4" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:AF1"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>